<commit_message>
feat: add the threats to the risk datawizard import
</commit_message>
<xml_diff>
--- a/backend/data_wizard/import_templates/risk_assessment_template.xlsx
+++ b/backend/data_wizard/import_templates/risk_assessment_template.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="13.5" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -484,6 +484,7 @@
     <col width="13.6640625" bestFit="1" customWidth="1" min="13" max="13"/>
     <col width="12.5" bestFit="1" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -567,6 +568,11 @@
           <t>assets</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>threats</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -626,6 +632,12 @@
 database server</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>ICT-001
+ICT-002</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -772,6 +784,11 @@
       <c r="P5" t="inlineStr">
         <is>
           <t>customer portal</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>ICT-003</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add threats to risk scenarios import (#5017)
* feat: add the threats to the risk datawizard import

* fix(data-wizard): resolve risk threats within the assessment's domain hierarchy

* fix(export): write threat ref_ids in risk assessment exports

* docs

* fix

* fix regression in test harness

---------

Co-authored-by: Eric <71850047+eric-intuitem@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/backend/data_wizard/import_templates/risk_assessment_template.xlsx
+++ b/backend/data_wizard/import_templates/risk_assessment_template.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="13.5" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -484,6 +484,7 @@
     <col width="13.6640625" bestFit="1" customWidth="1" min="13" max="13"/>
     <col width="12.5" bestFit="1" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -567,6 +568,11 @@
           <t>assets</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>threats</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -626,6 +632,12 @@
 database server</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>ICT-001
+ICT-002</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -772,6 +784,11 @@
       <c r="P5" t="inlineStr">
         <is>
           <t>customer portal</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>ICT-003</t>
         </is>
       </c>
     </row>

</xml_diff>